<commit_message>
Combining TEMPEST porewater data
</commit_message>
<xml_diff>
--- a/processing_scripts/pH/Raw Data/Data from Google Drive/TEMPEST_Porewater_pH.xlsx
+++ b/processing_scripts/pH/Raw Data/Data from Google Drive/TEMPEST_Porewater_pH.xlsx
@@ -15,10 +15,10 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author>tc={85b68696-62db-49d1-8d8f-238b2ef070a4}</author>
+    <author>tc={20850909-8e9e-496b-9d40-84713a0d74c8}</author>
   </authors>
   <commentList>
-    <comment authorId="0" xr:uid="{85b68696-62db-49d1-8d8f-238b2ef070a4}" ref="I229">
+    <comment authorId="0" xr:uid="{20850909-8e9e-496b-9d40-84713a0d74c8}" ref="I229">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -487,8 +487,8 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <x18tc:person displayName="Alice Stearns" id="{35327cca-4556-43ed-8439-dfb0e6013219}" providerId="google-sheets"/>
-  <x18tc:person displayName="Allison Myers-Pigg" id="{03796e49-00e4-416f-94b0-37669ac34825}" providerId="google-sheets"/>
+  <x18tc:person displayName="Alice Stearns" id="{a97089b9-b53a-42a4-9359-d280c423bf7f}" providerId="google-sheets"/>
+  <x18tc:person displayName="Allison Myers-Pigg" id="{93ab5e15-0f93-448d-b507-8791b2b82e09}" providerId="google-sheets"/>
 </x18tc:personList>
 </file>
 
@@ -688,10 +688,10 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="I229" dT="2024-12-17T16:39:13.00" personId="{03796e49-00e4-416f-94b0-37669ac34825}" id="{85b68696-62db-49d1-8d8f-238b2ef070a4}" done="1">
+  <x18tc:threadedComment ref="I229" dT="2024-12-17T16:39:13.00" personId="{93ab5e15-0f93-448d-b507-8791b2b82e09}" id="{20850909-8e9e-496b-9d40-84713a0d74c8}" done="1">
     <x18tc:text xml:space="preserve">Seems like all of these should be mS</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="I229" dT="2024-12-17T17:47:18.00" personId="{35327cca-4556-43ed-8439-dfb0e6013219}" id="{ef125f90-51dc-484e-a45c-a8523140b106}" parentId="{85b68696-62db-49d1-8d8f-238b2ef070a4}">
+  <x18tc:threadedComment ref="I229" dT="2024-12-17T17:47:18.00" personId="{a97089b9-b53a-42a4-9359-d280c423bf7f}" id="{b71b7b8c-c217-4620-8898-423e64fa90b7}" parentId="{20850909-8e9e-496b-9d40-84713a0d74c8}">
     <x18tc:text xml:space="preserve">I agree. It may have just been written down wrong on the field sheet</x18tc:text>
   </x18tc:threadedComment>
 </x18tc:ThreadedComments>

</xml_diff>